<commit_message>
Bug fixed in training_loss, working on multistart
</commit_message>
<xml_diff>
--- a/data/STEMI_merged.xlsx
+++ b/data/STEMI_merged.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\PHD_Projects\MechanisticAI\MechanisticsAI_julia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA6D2660-7983-4EB0-B5B1-6BB392306D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F66FFA-2AC7-4947-991A-5C537AE2CB9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28725" yWindow="2100" windowWidth="21600" windowHeight="12585" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4020" yWindow="2655" windowWidth="21600" windowHeight="12585" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tempi" sheetId="1" r:id="rId1"/>
@@ -26,8 +26,7 @@
     <sheet name="Misurazioni cleaned BK" sheetId="11" r:id="rId11"/>
     <sheet name="Patients ID" sheetId="12" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -801,7 +800,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normale 2" xfId="1" xr:uid="{E0239E55-A4D6-4209-B427-D3D8AE99B891}"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -6329,7 +6348,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10354,7 +10373,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="Z1:Z82 Z84:Z1048576 Y83">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26341,47 +26360,47 @@
         <v>4,045,272,425,970,752</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:26" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="14">
         <v>1.34</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="14">
         <v>3.11</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="14">
         <v>2.67</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="14">
         <v>2.78</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="14">
         <v>2.9</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="14">
         <v>2.13</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="14">
         <v>0.96899999999999997</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="14">
         <v>0.65800000000000003</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="14">
         <v>0.48299999999999998</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="14">
         <v>0.26800000000000002</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="14">
         <v>0.189</v>
       </c>
-      <c r="M21">
+      <c r="M21" s="14">
         <v>0.11799999999999999</v>
       </c>
-      <c r="Z21" t="str">
+      <c r="Z21" s="14" t="str">
         <f t="shared" si="0"/>
         <v>1,343,112,672,782,92,130,9690,6580,4830,2680,1890,118</v>
       </c>
@@ -30412,7 +30431,10 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="Z1:Z1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -38415,7 +38437,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="X71 Z1:Z70 Z72:Z82 Z84:Z96 Z98:Z1048576 X97 Y83">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>